<commit_message>
I have made 2 major chnages. Firstly I have written python code that will allow me to add any faculty to my database. Secondly I used R to convert my excell sheets containing the data I collected for the faculty of naturall science into a CSV file, this is becuase a CSV file will be a lot easier to work with in comparison to an excell sheet
</commit_message>
<xml_diff>
--- a/Faculties/Law/Programmes Law.xlsx
+++ b/Faculties/Law/Programmes Law.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d24d4a286855a075/Desktop/Team_6_repo/Team19/Faculties/Law/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B90C40EC-D302-4F5C-A634-A0A371EAEAB0}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7F07E22-673D-4C0C-AC1D-8F69BB265AF1}"/>
   <bookViews>
-    <workbookView xWindow="11352" yWindow="2616" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11100" yWindow="1104" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,6 @@
     <t>Abbreviation</t>
   </si>
   <si>
-    <t>Duration</t>
-  </si>
-  <si>
     <t>Bachelor of Laws</t>
   </si>
   <si>
@@ -48,30 +45,18 @@
     <t>4 years</t>
   </si>
   <si>
-    <t>Bachelor of Laws (Extended Curriculum Programme)</t>
-  </si>
-  <si>
-    <t>LLB (ECP)</t>
-  </si>
-  <si>
     <t>5 years</t>
   </si>
   <si>
     <t>Bachelor of Arts in Law</t>
   </si>
   <si>
-    <t>BA (Law)</t>
-  </si>
-  <si>
     <t>3 years</t>
   </si>
   <si>
     <t>Bachelor of Commerce in Law</t>
   </si>
   <si>
-    <t>BCom (Law)</t>
-  </si>
-  <si>
     <t>Master of Laws (Structured)</t>
   </si>
   <si>
@@ -93,18 +78,12 @@
     <t>Master of Laws in International Trade, Investment and Business Law</t>
   </si>
   <si>
-    <t>LLM (International Trade, Investment and Business Law)</t>
-  </si>
-  <si>
     <t>1 year full-time</t>
   </si>
   <si>
     <t>Master of Laws in Legal Pluralism and Family Law (Thesis)</t>
   </si>
   <si>
-    <t>LLM (Legal Pluralism and Family Law)</t>
-  </si>
-  <si>
     <t>Master of Laws in Legal Pluralism and Family Law (Structured)</t>
   </si>
   <si>
@@ -138,55 +117,76 @@
     <t>Advanced Diploma in Labour Law</t>
   </si>
   <si>
-    <t>AdvDip (Labour Law)</t>
-  </si>
-  <si>
     <t>Postgraduate Diploma in Environmental Law and Management</t>
   </si>
   <si>
     <t>7712 (FT) / 7713 (PT)</t>
   </si>
   <si>
-    <t>PGDip (Environmental Law and Management)</t>
-  </si>
-  <si>
     <t>Postgraduate Diploma in Fintech Law and Regulation</t>
   </si>
   <si>
     <t>7702 (FT) / 7703 (PT)</t>
   </si>
   <si>
-    <t>PGDip (Fintech Law and Regulation)</t>
-  </si>
-  <si>
     <t>Postgraduate Diploma in Labour Law</t>
   </si>
   <si>
-    <t>PGDip (Labour Law)</t>
-  </si>
-  <si>
     <t>Postgraduate Diploma in Public Law</t>
   </si>
   <si>
-    <t>PGDip (Public Law)</t>
-  </si>
-  <si>
     <t>Postgraduate Diploma in Tax Law</t>
   </si>
   <si>
     <t>7721 (FT) / 7722 (PT)</t>
   </si>
   <si>
-    <t>PGDip (Tax Law)</t>
-  </si>
-  <si>
     <t>Higher Certificate in Forensic Examination</t>
   </si>
   <si>
-    <t>HCert (Forensic Examination)</t>
-  </si>
-  <si>
     <t>1 year part-time</t>
+  </si>
+  <si>
+    <t>BA Law</t>
+  </si>
+  <si>
+    <t>BCom Law</t>
+  </si>
+  <si>
+    <t>LLM International Trade, Investment and Business Law</t>
+  </si>
+  <si>
+    <t>LLM Legal Pluralism and Family Law</t>
+  </si>
+  <si>
+    <t>AdvDip Labour Law</t>
+  </si>
+  <si>
+    <t>PGDip Environmental Law and Management</t>
+  </si>
+  <si>
+    <t>PGDip Fintech Law and Regulation</t>
+  </si>
+  <si>
+    <t>PGDip Labour Law</t>
+  </si>
+  <si>
+    <t>PGDip Public Law</t>
+  </si>
+  <si>
+    <t>PGDip Tax Law</t>
+  </si>
+  <si>
+    <t>HCert Forensic Examination</t>
+  </si>
+  <si>
+    <t>Bachelor of Laws Extended Curriculum Programme</t>
+  </si>
+  <si>
+    <t>Duration Years</t>
+  </si>
+  <si>
+    <t>LLB-ECP</t>
   </si>
 </sst>
 </file>
@@ -258,6 +258,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -532,7 +536,7 @@
     <col min="4" max="4" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -543,315 +547,315 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
       </c>
       <c r="B2" s="2">
         <v>7162</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="B3" s="2">
         <v>7172</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4" s="2">
         <v>7221</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="78" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2">
         <v>7211</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2">
         <v>7801</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>7821</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="78" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2">
         <v>7822</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="78" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="156" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="B9" s="2">
         <v>7811</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="124.8" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B10" s="2">
         <v>7831</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2">
         <v>7832</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2">
         <v>7871</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B13" s="2">
         <v>7860</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="109.2" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B14" s="2">
         <v>7861</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B15" s="2">
         <v>7921</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2">
         <v>7901</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2">
         <v>7311</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="156" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B20" s="2">
         <v>7701</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B21" s="2">
         <v>7711</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="D22" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="109.2" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B23" s="2">
         <v>7115</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>